<commit_message>
Refactor: Replace corporate branding with Global Markets Product Control Analytics across HTML reports, docs, and configs
</commit_message>
<xml_diff>
--- a/excel_client/ControlRunner.xlsx
+++ b/excel_client/ControlRunner.xlsx
@@ -526,7 +526,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="71" customWidth="1" min="2" max="2"/>
+    <col width="72" customWidth="1" min="2" max="2"/>
     <col width="21" customWidth="1" min="3" max="3"/>
     <col width="32" customWidth="1" min="4" max="4"/>
     <col width="28" customWidth="1" min="5" max="5"/>
@@ -539,7 +539,7 @@
     <row r="2">
       <c r="B2" s="1" t="inlineStr">
         <is>
-          <t>HSBC Product Control Analytics — Control Automation Service</t>
+          <t>Global Markets Product Control Analytics — Control Automation Service</t>
         </is>
       </c>
     </row>

</xml_diff>